<commit_message>
feat(ahp): enhance AHP module with new API endpoints and UI improvements
- Added new API endpoints for demand updates and AHP object management, including `PATCH` and `POST` methods for approval and analysis creation.
- Updated README.md to reflect new API routes and usage instructions for AHP analysis.
- Improved user interface in AHP steps, including clearer navigation and enhanced descriptions for each stage of the analysis process.
- Refined terminology in the AHP module, changing references from "matriz" to "tabela" for consistency.
- Enhanced JavaScript functionality for live metrics updates during pairwise comparisons, improving user feedback and interaction.
</commit_message>
<xml_diff>
--- a/data/Modelo_Matriz_Criterios_Premissas_Analise.xlsx
+++ b/data/Modelo_Matriz_Criterios_Premissas_Analise.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Matriz de Criterios e Premissas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tabela de Premissas e Critérios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="_Listas" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="Exemplo de preenchimento" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -2535,7 +2535,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INSTRUCOES DE PREENCHIMENTO — Matriz de Criterios e Premissas (Analise AHP)</t>
+          <t>INSTRUCOES DE PREENCHIMENTO — Tabela de Premissas e Criterios (Analise AHP)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -2551,7 +2551,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. Use a aba «Matriz de Criterios e Premissas» para cadastrar a etapa conceitual da sua analise.</t>
+          <t>1. Use a aba «Tabela de Premissas e Critérios» para cadastrar a etapa conceitual da sua analise.</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2610,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Exemplos reais (matriz de referencia PLI-SP) — abaixo:</t>
+          <t>Exemplos reais (tabela de referencia PLI-SP) — abaixo:</t>
         </is>
       </c>
     </row>

</xml_diff>